<commit_message>
Direct Write Excel for COMP-01 Day 6
</commit_message>
<xml_diff>
--- a/FM-MN-07_COMP-01.xlsx
+++ b/FM-MN-07_COMP-01.xlsx
@@ -1717,7 +1717,11 @@
       <c r="E6" s="25" t="inlineStr"/>
       <c r="F6" s="25" t="inlineStr"/>
       <c r="G6" s="25" t="inlineStr"/>
-      <c r="H6" s="25" t="inlineStr"/>
+      <c r="H6" s="25" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I6" s="25" t="inlineStr"/>
       <c r="J6" s="25" t="inlineStr"/>
       <c r="K6" s="25" t="inlineStr"/>
@@ -1758,7 +1762,11 @@
       <c r="E7" s="25" t="inlineStr"/>
       <c r="F7" s="25" t="inlineStr"/>
       <c r="G7" s="25" t="inlineStr"/>
-      <c r="H7" s="25" t="inlineStr"/>
+      <c r="H7" s="25" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I7" s="25" t="inlineStr"/>
       <c r="J7" s="25" t="inlineStr"/>
       <c r="K7" s="25" t="inlineStr"/>
@@ -1799,7 +1807,11 @@
       <c r="E8" s="25" t="inlineStr"/>
       <c r="F8" s="25" t="inlineStr"/>
       <c r="G8" s="25" t="inlineStr"/>
-      <c r="H8" s="25" t="inlineStr"/>
+      <c r="H8" s="25" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I8" s="25" t="inlineStr"/>
       <c r="J8" s="25" t="inlineStr"/>
       <c r="K8" s="25" t="inlineStr"/>
@@ -1840,7 +1852,11 @@
       <c r="E9" s="25" t="inlineStr"/>
       <c r="F9" s="25" t="inlineStr"/>
       <c r="G9" s="25" t="inlineStr"/>
-      <c r="H9" s="25" t="inlineStr"/>
+      <c r="H9" s="25" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I9" s="25" t="inlineStr"/>
       <c r="J9" s="25" t="inlineStr"/>
       <c r="K9" s="25" t="inlineStr"/>
@@ -1881,7 +1897,11 @@
       <c r="E10" s="25" t="inlineStr"/>
       <c r="F10" s="25" t="inlineStr"/>
       <c r="G10" s="25" t="inlineStr"/>
-      <c r="H10" s="25" t="inlineStr"/>
+      <c r="H10" s="25" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I10" s="25" t="inlineStr"/>
       <c r="J10" s="25" t="inlineStr"/>
       <c r="K10" s="25" t="inlineStr"/>
@@ -1916,7 +1936,11 @@
       <c r="E11" s="36" t="inlineStr"/>
       <c r="F11" s="36" t="inlineStr"/>
       <c r="G11" s="36" t="inlineStr"/>
-      <c r="H11" s="36" t="inlineStr"/>
+      <c r="H11" s="38" t="inlineStr">
+        <is>
+          <t>Chit shar</t>
+        </is>
+      </c>
       <c r="I11" s="36" t="inlineStr"/>
       <c r="J11" s="36" t="inlineStr"/>
       <c r="K11" s="36" t="inlineStr"/>
@@ -2099,8 +2123,8 @@
     <mergeCell ref="Y11:Y12"/>
     <mergeCell ref="J11:J12"/>
     <mergeCell ref="AG11:AG12"/>
+    <mergeCell ref="B16:AG16"/>
     <mergeCell ref="P11:P12"/>
-    <mergeCell ref="B16:AG16"/>
     <mergeCell ref="AB2:AG2"/>
     <mergeCell ref="AC18:AG18"/>
     <mergeCell ref="K11:K12"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for COMP-01 Day 7
</commit_message>
<xml_diff>
--- a/FM-MN-07_COMP-01.xlsx
+++ b/FM-MN-07_COMP-01.xlsx
@@ -1722,7 +1722,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I6" s="25" t="inlineStr"/>
+      <c r="I6" s="25" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J6" s="25" t="inlineStr"/>
       <c r="K6" s="25" t="inlineStr"/>
       <c r="L6" s="25" t="inlineStr"/>
@@ -1767,7 +1771,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I7" s="25" t="inlineStr"/>
+      <c r="I7" s="25" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J7" s="25" t="inlineStr"/>
       <c r="K7" s="25" t="inlineStr"/>
       <c r="L7" s="25" t="inlineStr"/>
@@ -1812,7 +1820,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I8" s="25" t="inlineStr"/>
+      <c r="I8" s="25" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J8" s="25" t="inlineStr"/>
       <c r="K8" s="25" t="inlineStr"/>
       <c r="L8" s="25" t="inlineStr"/>
@@ -1857,7 +1869,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I9" s="25" t="inlineStr"/>
+      <c r="I9" s="25" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J9" s="25" t="inlineStr"/>
       <c r="K9" s="25" t="inlineStr"/>
       <c r="L9" s="25" t="inlineStr"/>
@@ -1902,7 +1918,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I10" s="25" t="inlineStr"/>
+      <c r="I10" s="25" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J10" s="25" t="inlineStr"/>
       <c r="K10" s="25" t="inlineStr"/>
       <c r="L10" s="25" t="inlineStr"/>
@@ -1941,7 +1961,11 @@
           <t>Chit shar</t>
         </is>
       </c>
-      <c r="I11" s="36" t="inlineStr"/>
+      <c r="I11" s="38" t="inlineStr">
+        <is>
+          <t>Chit shar</t>
+        </is>
+      </c>
       <c r="J11" s="36" t="inlineStr"/>
       <c r="K11" s="36" t="inlineStr"/>
       <c r="L11" s="36" t="inlineStr"/>
@@ -2123,8 +2147,8 @@
     <mergeCell ref="Y11:Y12"/>
     <mergeCell ref="J11:J12"/>
     <mergeCell ref="AG11:AG12"/>
+    <mergeCell ref="P11:P12"/>
     <mergeCell ref="B16:AG16"/>
-    <mergeCell ref="P11:P12"/>
     <mergeCell ref="AB2:AG2"/>
     <mergeCell ref="AC18:AG18"/>
     <mergeCell ref="K11:K12"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for COMP-01 Day 8
</commit_message>
<xml_diff>
--- a/FM-MN-07_COMP-01.xlsx
+++ b/FM-MN-07_COMP-01.xlsx
@@ -1730,7 +1730,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J6" s="25" t="inlineStr"/>
+      <c r="J6" s="25" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K6" s="25" t="inlineStr"/>
       <c r="L6" s="25" t="inlineStr"/>
       <c r="M6" s="25" t="inlineStr"/>
@@ -1779,7 +1783,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J7" s="25" t="inlineStr"/>
+      <c r="J7" s="25" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K7" s="25" t="inlineStr"/>
       <c r="L7" s="25" t="inlineStr"/>
       <c r="M7" s="25" t="inlineStr"/>
@@ -1828,7 +1836,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J8" s="25" t="inlineStr"/>
+      <c r="J8" s="25" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K8" s="25" t="inlineStr"/>
       <c r="L8" s="25" t="inlineStr"/>
       <c r="M8" s="25" t="inlineStr"/>
@@ -1877,7 +1889,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J9" s="25" t="inlineStr"/>
+      <c r="J9" s="25" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K9" s="25" t="inlineStr"/>
       <c r="L9" s="25" t="inlineStr"/>
       <c r="M9" s="25" t="inlineStr"/>
@@ -1926,7 +1942,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J10" s="25" t="inlineStr"/>
+      <c r="J10" s="25" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K10" s="25" t="inlineStr"/>
       <c r="L10" s="25" t="inlineStr"/>
       <c r="M10" s="25" t="inlineStr"/>
@@ -1969,7 +1989,11 @@
           <t>Chit shar</t>
         </is>
       </c>
-      <c r="J11" s="36" t="inlineStr"/>
+      <c r="J11" s="38" t="inlineStr">
+        <is>
+          <t>Chit shar</t>
+        </is>
+      </c>
       <c r="K11" s="36" t="inlineStr"/>
       <c r="L11" s="36" t="inlineStr"/>
       <c r="M11" s="36" t="inlineStr"/>
@@ -2154,8 +2178,8 @@
     <mergeCell ref="Y11:Y12"/>
     <mergeCell ref="J11:J12"/>
     <mergeCell ref="AG11:AG12"/>
+    <mergeCell ref="P11:P12"/>
     <mergeCell ref="B16:AG16"/>
-    <mergeCell ref="P11:P12"/>
     <mergeCell ref="AB2:AG2"/>
     <mergeCell ref="AC18:AG18"/>
     <mergeCell ref="K11:K12"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for COMP-01 Day 10
</commit_message>
<xml_diff>
--- a/FM-MN-07_COMP-01.xlsx
+++ b/FM-MN-07_COMP-01.xlsx
@@ -1736,7 +1736,11 @@
         </is>
       </c>
       <c r="K6" s="25" t="inlineStr"/>
-      <c r="L6" s="25" t="inlineStr"/>
+      <c r="L6" s="25" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M6" s="25" t="inlineStr"/>
       <c r="N6" s="25" t="inlineStr"/>
       <c r="O6" s="25" t="inlineStr"/>
@@ -1789,7 +1793,11 @@
         </is>
       </c>
       <c r="K7" s="25" t="inlineStr"/>
-      <c r="L7" s="25" t="inlineStr"/>
+      <c r="L7" s="25" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M7" s="25" t="inlineStr"/>
       <c r="N7" s="25" t="inlineStr"/>
       <c r="O7" s="25" t="inlineStr"/>
@@ -1842,7 +1850,11 @@
         </is>
       </c>
       <c r="K8" s="25" t="inlineStr"/>
-      <c r="L8" s="25" t="inlineStr"/>
+      <c r="L8" s="25" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M8" s="25" t="inlineStr"/>
       <c r="N8" s="25" t="inlineStr"/>
       <c r="O8" s="25" t="inlineStr"/>
@@ -1895,7 +1907,11 @@
         </is>
       </c>
       <c r="K9" s="25" t="inlineStr"/>
-      <c r="L9" s="25" t="inlineStr"/>
+      <c r="L9" s="25" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M9" s="25" t="inlineStr"/>
       <c r="N9" s="25" t="inlineStr"/>
       <c r="O9" s="25" t="inlineStr"/>
@@ -1948,7 +1964,11 @@
         </is>
       </c>
       <c r="K10" s="25" t="inlineStr"/>
-      <c r="L10" s="25" t="inlineStr"/>
+      <c r="L10" s="25" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M10" s="25" t="inlineStr"/>
       <c r="N10" s="25" t="inlineStr"/>
       <c r="O10" s="25" t="inlineStr"/>
@@ -1995,7 +2015,11 @@
         </is>
       </c>
       <c r="K11" s="36" t="inlineStr"/>
-      <c r="L11" s="36" t="inlineStr"/>
+      <c r="L11" s="38" t="inlineStr">
+        <is>
+          <t>Chit shar</t>
+        </is>
+      </c>
       <c r="M11" s="36" t="inlineStr"/>
       <c r="N11" s="36" t="inlineStr"/>
       <c r="O11" s="36" t="inlineStr"/>
@@ -2178,8 +2202,8 @@
     <mergeCell ref="Y11:Y12"/>
     <mergeCell ref="J11:J12"/>
     <mergeCell ref="AG11:AG12"/>
+    <mergeCell ref="B16:AG16"/>
     <mergeCell ref="P11:P12"/>
-    <mergeCell ref="B16:AG16"/>
     <mergeCell ref="AB2:AG2"/>
     <mergeCell ref="AC18:AG18"/>
     <mergeCell ref="K11:K12"/>

</xml_diff>